<commit_message>
Error Resolved for ClinicDB
</commit_message>
<xml_diff>
--- a/MK_UNet_ClinicDB_Results/All_Runs_Summary_Polyp.xlsx
+++ b/MK_UNet_ClinicDB_Results/All_Runs_Summary_Polyp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\MK_UNet_Replication_Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Study Material\✅✅Professor_Mail\Mostafijur_Rahman\MK-UNet\MK_UNet_ClinicDB_Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09D9974-942A-46A9-9673-B0574167FDE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6B1A76-5DE4-4921-BAB0-B88739C3ADE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-10095" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>